<commit_message>
Update Bàn giao linh kiẹn X-Force Vnet 052026 - kiểm tra lại - Copy.xlsx
</commit_message>
<xml_diff>
--- a/2. Báo cáo - giấy tờ/1. Báo cáo/Bàn giao/Bàn giao linh kiẹn X-Force Vnet 052026 - kiểm tra lại - Copy.xlsx
+++ b/2. Báo cáo - giấy tờ/1. Báo cáo/Bàn giao/Bàn giao linh kiẹn X-Force Vnet 052026 - kiểm tra lại - Copy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TungNM\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\2. Báo cáo - giấy tờ\1. Báo cáo\Bàn giao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460CC8FF-A55E-427A-9269-BA95A212E87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AB6BE13-3FB4-451F-ABAC-5BB75519F6CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -809,6 +809,24 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -825,24 +843,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1271,58 +1271,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="30" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
     </row>
     <row r="2" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="32"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="31" t="s">
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="32"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="31" t="s">
+      <c r="A3" s="26"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
     </row>
     <row r="4" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="33"/>
-      <c r="B4" s="33"/>
-      <c r="C4" s="31" t="s">
+      <c r="A4" s="27"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
     </row>
     <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
     </row>
     <row r="6" spans="1:5" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="22"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="24"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
@@ -1390,7 +1390,7 @@
       <c r="D12" s="11">
         <v>489</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="33" t="s">
         <v>143</v>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       <c r="D13" s="11">
         <v>488</v>
       </c>
-      <c r="E13" s="27"/>
+      <c r="E13" s="33"/>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
@@ -1422,7 +1422,7 @@
       <c r="D14" s="21">
         <v>3465</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="33"/>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
@@ -1437,7 +1437,7 @@
       <c r="D15" s="11">
         <v>990</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="33"/>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
@@ -1452,7 +1452,7 @@
       <c r="D16" s="11">
         <v>990</v>
       </c>
-      <c r="E16" s="27"/>
+      <c r="E16" s="33"/>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
@@ -1467,7 +1467,7 @@
       <c r="D17" s="11">
         <v>2475</v>
       </c>
-      <c r="E17" s="27"/>
+      <c r="E17" s="33"/>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
@@ -1482,7 +1482,7 @@
       <c r="D18" s="11">
         <v>5445</v>
       </c>
-      <c r="E18" s="27"/>
+      <c r="E18" s="33"/>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
@@ -1497,7 +1497,7 @@
       <c r="D19" s="11">
         <v>990</v>
       </c>
-      <c r="E19" s="27"/>
+      <c r="E19" s="33"/>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
@@ -1512,7 +1512,7 @@
       <c r="D20" s="11">
         <v>495</v>
       </c>
-      <c r="E20" s="27"/>
+      <c r="E20" s="33"/>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="10">
@@ -1527,7 +1527,7 @@
       <c r="D21" s="11">
         <v>40570</v>
       </c>
-      <c r="E21" s="27"/>
+      <c r="E21" s="33"/>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
@@ -1542,7 +1542,7 @@
       <c r="D22" s="21">
         <v>990</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="33"/>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
@@ -1557,7 +1557,7 @@
       <c r="D23" s="11">
         <v>495</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="33"/>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
@@ -1572,7 +1572,7 @@
       <c r="D24" s="21">
         <v>495</v>
       </c>
-      <c r="E24" s="27"/>
+      <c r="E24" s="33"/>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
@@ -1587,7 +1587,7 @@
       <c r="D25" s="11">
         <v>495</v>
       </c>
-      <c r="E25" s="27"/>
+      <c r="E25" s="33"/>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
@@ -1602,7 +1602,7 @@
       <c r="D26" s="11">
         <v>495</v>
       </c>
-      <c r="E26" s="27"/>
+      <c r="E26" s="33"/>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10">
@@ -1617,7 +1617,7 @@
       <c r="D27" s="11">
         <v>495</v>
       </c>
-      <c r="E27" s="27"/>
+      <c r="E27" s="33"/>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10">
@@ -1632,7 +1632,7 @@
       <c r="D28" s="11">
         <v>495</v>
       </c>
-      <c r="E28" s="27"/>
+      <c r="E28" s="33"/>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
@@ -1647,7 +1647,7 @@
       <c r="D29" s="11">
         <v>3945</v>
       </c>
-      <c r="E29" s="27"/>
+      <c r="E29" s="33"/>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
@@ -1662,7 +1662,7 @@
       <c r="D30" s="21">
         <v>13360</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="33"/>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
@@ -1677,7 +1677,7 @@
       <c r="D31" s="11">
         <v>1485</v>
       </c>
-      <c r="E31" s="27"/>
+      <c r="E31" s="33"/>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="10">
@@ -1692,7 +1692,7 @@
       <c r="D32" s="11">
         <v>3960</v>
       </c>
-      <c r="E32" s="27"/>
+      <c r="E32" s="33"/>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="10">
@@ -1707,7 +1707,7 @@
       <c r="D33" s="11">
         <v>495</v>
       </c>
-      <c r="E33" s="27"/>
+      <c r="E33" s="33"/>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="10">
@@ -1722,7 +1722,7 @@
       <c r="D34" s="21">
         <v>495</v>
       </c>
-      <c r="E34" s="27"/>
+      <c r="E34" s="33"/>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="10">
@@ -1737,7 +1737,7 @@
       <c r="D35" s="11">
         <v>990</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="33"/>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="10">
@@ -1752,7 +1752,7 @@
       <c r="D36" s="11">
         <v>495</v>
       </c>
-      <c r="E36" s="27"/>
+      <c r="E36" s="33"/>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10">
@@ -1767,7 +1767,7 @@
       <c r="D37" s="11">
         <v>495</v>
       </c>
-      <c r="E37" s="27"/>
+      <c r="E37" s="33"/>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10">
@@ -1782,7 +1782,7 @@
       <c r="D38" s="11">
         <v>495</v>
       </c>
-      <c r="E38" s="27"/>
+      <c r="E38" s="33"/>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10">
@@ -1797,7 +1797,7 @@
       <c r="D39" s="11">
         <v>990</v>
       </c>
-      <c r="E39" s="27"/>
+      <c r="E39" s="33"/>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10">
@@ -1812,7 +1812,7 @@
       <c r="D40" s="11">
         <v>990</v>
       </c>
-      <c r="E40" s="27"/>
+      <c r="E40" s="33"/>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="10">
@@ -1827,7 +1827,7 @@
       <c r="D41" s="21">
         <v>495</v>
       </c>
-      <c r="E41" s="27"/>
+      <c r="E41" s="33"/>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="10">
@@ -1842,7 +1842,7 @@
       <c r="D42" s="11">
         <v>495</v>
       </c>
-      <c r="E42" s="27"/>
+      <c r="E42" s="33"/>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10">
@@ -1857,7 +1857,7 @@
       <c r="D43" s="11">
         <v>495</v>
       </c>
-      <c r="E43" s="27"/>
+      <c r="E43" s="33"/>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="10">
@@ -1872,7 +1872,7 @@
       <c r="D44" s="11">
         <v>985</v>
       </c>
-      <c r="E44" s="27"/>
+      <c r="E44" s="33"/>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10">
@@ -1887,7 +1887,7 @@
       <c r="D45" s="11">
         <v>495</v>
       </c>
-      <c r="E45" s="27"/>
+      <c r="E45" s="33"/>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10">
@@ -1902,7 +1902,7 @@
       <c r="D46" s="11">
         <v>495</v>
       </c>
-      <c r="E46" s="27"/>
+      <c r="E46" s="33"/>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10">
@@ -1917,7 +1917,7 @@
       <c r="D47" s="21">
         <v>500</v>
       </c>
-      <c r="E47" s="27"/>
+      <c r="E47" s="33"/>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10">
@@ -1932,7 +1932,7 @@
       <c r="D48" s="11">
         <v>495</v>
       </c>
-      <c r="E48" s="27"/>
+      <c r="E48" s="33"/>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10">
@@ -1947,7 +1947,7 @@
       <c r="D49" s="11">
         <v>495</v>
       </c>
-      <c r="E49" s="27"/>
+      <c r="E49" s="33"/>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10">
@@ -1962,7 +1962,7 @@
       <c r="D50" s="21">
         <v>4445</v>
       </c>
-      <c r="E50" s="27"/>
+      <c r="E50" s="33"/>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10">
@@ -1977,7 +1977,7 @@
       <c r="D51" s="11">
         <v>2970</v>
       </c>
-      <c r="E51" s="27"/>
+      <c r="E51" s="33"/>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="10">
@@ -1992,7 +1992,7 @@
       <c r="D52" s="11">
         <v>495</v>
       </c>
-      <c r="E52" s="27"/>
+      <c r="E52" s="33"/>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10">
@@ -2007,7 +2007,7 @@
       <c r="D53" s="11">
         <v>495</v>
       </c>
-      <c r="E53" s="27"/>
+      <c r="E53" s="33"/>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="10">
@@ -2022,7 +2022,7 @@
       <c r="D54" s="11">
         <v>490</v>
       </c>
-      <c r="E54" s="27"/>
+      <c r="E54" s="33"/>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10">
@@ -2037,7 +2037,7 @@
       <c r="D55" s="11">
         <v>6915</v>
       </c>
-      <c r="E55" s="27"/>
+      <c r="E55" s="33"/>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="10">
@@ -2052,7 +2052,7 @@
       <c r="D56" s="11">
         <v>495</v>
       </c>
-      <c r="E56" s="27"/>
+      <c r="E56" s="33"/>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="10">
@@ -2067,7 +2067,7 @@
       <c r="D57" s="11">
         <v>2475</v>
       </c>
-      <c r="E57" s="27"/>
+      <c r="E57" s="33"/>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="10">
@@ -2082,7 +2082,7 @@
       <c r="D58" s="11">
         <v>990</v>
       </c>
-      <c r="E58" s="27"/>
+      <c r="E58" s="33"/>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="10">
@@ -2097,7 +2097,7 @@
       <c r="D59" s="11">
         <v>495</v>
       </c>
-      <c r="E59" s="27"/>
+      <c r="E59" s="33"/>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="10">
@@ -2112,7 +2112,7 @@
       <c r="D60" s="11">
         <v>495</v>
       </c>
-      <c r="E60" s="27"/>
+      <c r="E60" s="33"/>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="10">
@@ -2127,7 +2127,7 @@
       <c r="D61" s="11">
         <v>990</v>
       </c>
-      <c r="E61" s="27"/>
+      <c r="E61" s="33"/>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="10">
@@ -2142,7 +2142,7 @@
       <c r="D62" s="11">
         <v>4950</v>
       </c>
-      <c r="E62" s="27"/>
+      <c r="E62" s="33"/>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="10">
@@ -2157,7 +2157,7 @@
       <c r="D63" s="11">
         <v>2970</v>
       </c>
-      <c r="E63" s="27"/>
+      <c r="E63" s="33"/>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="10">
@@ -2172,7 +2172,7 @@
       <c r="D64" s="11">
         <v>6435</v>
       </c>
-      <c r="E64" s="27"/>
+      <c r="E64" s="33"/>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="10">
@@ -2187,7 +2187,7 @@
       <c r="D65" s="11">
         <v>990</v>
       </c>
-      <c r="E65" s="27"/>
+      <c r="E65" s="33"/>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="10" t="s">
@@ -2202,7 +2202,7 @@
       <c r="D66" s="11">
         <v>495</v>
       </c>
-      <c r="E66" s="27"/>
+      <c r="E66" s="33"/>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="10">
@@ -2217,7 +2217,7 @@
       <c r="D67" s="11">
         <v>990</v>
       </c>
-      <c r="E67" s="27"/>
+      <c r="E67" s="33"/>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="10">
@@ -2232,7 +2232,7 @@
       <c r="D68" s="11">
         <v>495</v>
       </c>
-      <c r="E68" s="27"/>
+      <c r="E68" s="33"/>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A69" s="10">
@@ -2247,7 +2247,7 @@
       <c r="D69" s="11">
         <v>495</v>
       </c>
-      <c r="E69" s="27"/>
+      <c r="E69" s="33"/>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="10">
@@ -2262,7 +2262,7 @@
       <c r="D70" s="11">
         <v>1980</v>
       </c>
-      <c r="E70" s="27"/>
+      <c r="E70" s="33"/>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="10">
@@ -2277,7 +2277,7 @@
       <c r="D71" s="11">
         <v>1485</v>
       </c>
-      <c r="E71" s="27"/>
+      <c r="E71" s="33"/>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="10">
@@ -2292,7 +2292,7 @@
       <c r="D72" s="11">
         <v>990</v>
       </c>
-      <c r="E72" s="27"/>
+      <c r="E72" s="33"/>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="10">
@@ -2307,7 +2307,7 @@
       <c r="D73" s="11">
         <v>495</v>
       </c>
-      <c r="E73" s="27"/>
+      <c r="E73" s="33"/>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="10">
@@ -2322,7 +2322,7 @@
       <c r="D74" s="11">
         <v>495</v>
       </c>
-      <c r="E74" s="27"/>
+      <c r="E74" s="33"/>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="10">
@@ -2337,7 +2337,7 @@
       <c r="D75" s="11">
         <v>495</v>
       </c>
-      <c r="E75" s="27"/>
+      <c r="E75" s="33"/>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="10">
@@ -2352,7 +2352,7 @@
       <c r="D76" s="11">
         <v>495</v>
       </c>
-      <c r="E76" s="27"/>
+      <c r="E76" s="33"/>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="10">
@@ -2367,7 +2367,7 @@
       <c r="D77" s="11">
         <v>495</v>
       </c>
-      <c r="E77" s="27"/>
+      <c r="E77" s="33"/>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="10">
@@ -2382,7 +2382,7 @@
       <c r="D78" s="11">
         <v>495</v>
       </c>
-      <c r="E78" s="27"/>
+      <c r="E78" s="33"/>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="10">
@@ -2397,7 +2397,7 @@
       <c r="D79" s="11">
         <v>495</v>
       </c>
-      <c r="E79" s="27"/>
+      <c r="E79" s="33"/>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="10">
@@ -2412,7 +2412,7 @@
       <c r="D80" s="11">
         <v>495</v>
       </c>
-      <c r="E80" s="27"/>
+      <c r="E80" s="33"/>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="10">
@@ -2427,7 +2427,7 @@
       <c r="D81" s="11">
         <v>990</v>
       </c>
-      <c r="E81" s="27"/>
+      <c r="E81" s="33"/>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="10">
@@ -2442,7 +2442,7 @@
       <c r="D82" s="21">
         <v>495</v>
       </c>
-      <c r="E82" s="27"/>
+      <c r="E82" s="33"/>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="10">
@@ -2457,7 +2457,7 @@
       <c r="D83" s="11">
         <v>495</v>
       </c>
-      <c r="E83" s="27"/>
+      <c r="E83" s="33"/>
     </row>
     <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="10">
@@ -2472,7 +2472,7 @@
       <c r="D84" s="11">
         <v>1480</v>
       </c>
-      <c r="E84" s="27"/>
+      <c r="E84" s="33"/>
     </row>
     <row r="85" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="10">
@@ -2487,7 +2487,7 @@
       <c r="D85" s="11">
         <v>1485</v>
       </c>
-      <c r="E85" s="27"/>
+      <c r="E85" s="33"/>
     </row>
     <row r="86" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="10">
@@ -2502,7 +2502,7 @@
       <c r="D86" s="11">
         <v>495</v>
       </c>
-      <c r="E86" s="27"/>
+      <c r="E86" s="33"/>
     </row>
     <row r="87" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="10">
@@ -2517,7 +2517,7 @@
       <c r="D87" s="11">
         <v>3455</v>
       </c>
-      <c r="E87" s="27"/>
+      <c r="E87" s="33"/>
     </row>
     <row r="88" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="10">
@@ -2532,7 +2532,7 @@
       <c r="D88" s="11">
         <v>495</v>
       </c>
-      <c r="E88" s="27"/>
+      <c r="E88" s="33"/>
     </row>
     <row r="89" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="10">
@@ -2547,7 +2547,7 @@
       <c r="D89" s="11">
         <v>2970</v>
       </c>
-      <c r="E89" s="27"/>
+      <c r="E89" s="33"/>
     </row>
     <row r="90" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="10">
@@ -2562,7 +2562,7 @@
       <c r="D90" s="11">
         <v>495</v>
       </c>
-      <c r="E90" s="27"/>
+      <c r="E90" s="33"/>
     </row>
     <row r="91" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="10">
@@ -2577,7 +2577,7 @@
       <c r="D91" s="11">
         <v>495</v>
       </c>
-      <c r="E91" s="27"/>
+      <c r="E91" s="33"/>
     </row>
     <row r="92" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="10">
@@ -2592,7 +2592,7 @@
       <c r="D92" s="11">
         <v>4950</v>
       </c>
-      <c r="E92" s="27"/>
+      <c r="E92" s="33"/>
     </row>
     <row r="93" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="10">
@@ -2607,7 +2607,7 @@
       <c r="D93" s="11">
         <v>495</v>
       </c>
-      <c r="E93" s="27"/>
+      <c r="E93" s="33"/>
     </row>
     <row r="94" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A94" s="10">
@@ -2622,7 +2622,7 @@
       <c r="D94" s="21">
         <v>21090</v>
       </c>
-      <c r="E94" s="27"/>
+      <c r="E94" s="33"/>
     </row>
     <row r="95" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="10">
@@ -2637,7 +2637,7 @@
       <c r="D95" s="11">
         <v>16805</v>
       </c>
-      <c r="E95" s="27"/>
+      <c r="E95" s="33"/>
     </row>
     <row r="96" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="10">
@@ -2652,7 +2652,7 @@
       <c r="D96" s="11">
         <v>495</v>
       </c>
-      <c r="E96" s="27"/>
+      <c r="E96" s="33"/>
     </row>
     <row r="97" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A97" s="10">
@@ -2667,7 +2667,7 @@
       <c r="D97" s="11">
         <v>495</v>
       </c>
-      <c r="E97" s="27"/>
+      <c r="E97" s="33"/>
     </row>
     <row r="98" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A98" s="10">
@@ -2682,7 +2682,7 @@
       <c r="D98" s="11">
         <v>990</v>
       </c>
-      <c r="E98" s="27"/>
+      <c r="E98" s="33"/>
     </row>
     <row r="99" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="10">
@@ -2697,7 +2697,7 @@
       <c r="D99" s="11">
         <v>495</v>
       </c>
-      <c r="E99" s="27"/>
+      <c r="E99" s="33"/>
     </row>
     <row r="100" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A100" s="10">
@@ -2712,7 +2712,7 @@
       <c r="D100" s="21">
         <v>500</v>
       </c>
-      <c r="E100" s="27"/>
+      <c r="E100" s="33"/>
     </row>
     <row r="101" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="10">
@@ -2727,7 +2727,7 @@
       <c r="D101" s="11">
         <v>495</v>
       </c>
-      <c r="E101" s="27"/>
+      <c r="E101" s="33"/>
     </row>
     <row r="102" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="10">
@@ -2742,7 +2742,7 @@
       <c r="D102" s="11">
         <v>2475</v>
       </c>
-      <c r="E102" s="27"/>
+      <c r="E102" s="33"/>
     </row>
     <row r="103" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="10">
@@ -2757,7 +2757,7 @@
       <c r="D103" s="11">
         <v>9385</v>
       </c>
-      <c r="E103" s="27"/>
+      <c r="E103" s="33"/>
     </row>
     <row r="104" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A104" s="10">
@@ -2772,7 +2772,7 @@
       <c r="D104" s="11">
         <v>495</v>
       </c>
-      <c r="E104" s="27"/>
+      <c r="E104" s="33"/>
     </row>
     <row r="105" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="10">
@@ -2787,7 +2787,7 @@
       <c r="D105" s="11">
         <v>495</v>
       </c>
-      <c r="E105" s="27"/>
+      <c r="E105" s="33"/>
     </row>
     <row r="106" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="10">
@@ -2802,7 +2802,7 @@
       <c r="D106" s="11">
         <v>495</v>
       </c>
-      <c r="E106" s="27"/>
+      <c r="E106" s="33"/>
     </row>
     <row r="107" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="10">
@@ -2817,7 +2817,7 @@
       <c r="D107" s="11">
         <v>495</v>
       </c>
-      <c r="E107" s="27"/>
+      <c r="E107" s="33"/>
     </row>
     <row r="108" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="10">
@@ -2832,7 +2832,7 @@
       <c r="D108" s="11">
         <v>7400</v>
       </c>
-      <c r="E108" s="27"/>
+      <c r="E108" s="33"/>
     </row>
     <row r="109" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A109" s="10">
@@ -2847,7 +2847,7 @@
       <c r="D109" s="11">
         <v>990</v>
       </c>
-      <c r="E109" s="27"/>
+      <c r="E109" s="33"/>
     </row>
     <row r="110" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="10">
@@ -2862,7 +2862,7 @@
       <c r="D110" s="11">
         <v>13365</v>
       </c>
-      <c r="E110" s="27"/>
+      <c r="E110" s="33"/>
     </row>
     <row r="111" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A111" s="10">
@@ -2877,7 +2877,7 @@
       <c r="D111" s="11">
         <v>495</v>
       </c>
-      <c r="E111" s="27"/>
+      <c r="E111" s="33"/>
     </row>
     <row r="112" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A112" s="10">
@@ -2892,7 +2892,7 @@
       <c r="D112" s="11">
         <v>990</v>
       </c>
-      <c r="E112" s="27"/>
+      <c r="E112" s="33"/>
     </row>
     <row r="113" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A113" s="10">
@@ -2907,7 +2907,7 @@
       <c r="D113" s="11">
         <v>10000</v>
       </c>
-      <c r="E113" s="27"/>
+      <c r="E113" s="33"/>
     </row>
     <row r="114" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A114" s="10">
@@ -2922,7 +2922,7 @@
       <c r="D114" s="11">
         <v>490</v>
       </c>
-      <c r="E114" s="27"/>
+      <c r="E114" s="33"/>
     </row>
     <row r="115" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A115" s="10">
@@ -2937,7 +2937,7 @@
       <c r="D115" s="11">
         <v>495</v>
       </c>
-      <c r="E115" s="27"/>
+      <c r="E115" s="33"/>
     </row>
     <row r="116" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A116" s="10">
@@ -2952,7 +2952,7 @@
       <c r="D116" s="11">
         <v>4450</v>
       </c>
-      <c r="E116" s="27"/>
+      <c r="E116" s="33"/>
     </row>
     <row r="117" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A117" s="10">
@@ -2967,7 +2967,7 @@
       <c r="D117" s="11">
         <v>1980</v>
       </c>
-      <c r="E117" s="27"/>
+      <c r="E117" s="33"/>
     </row>
     <row r="118" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A118" s="10">
@@ -2982,7 +2982,7 @@
       <c r="D118" s="11">
         <v>495</v>
       </c>
-      <c r="E118" s="27"/>
+      <c r="E118" s="33"/>
     </row>
     <row r="119" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A119" s="10">
@@ -2997,7 +2997,7 @@
       <c r="D119" s="21">
         <v>8420</v>
       </c>
-      <c r="E119" s="27"/>
+      <c r="E119" s="33"/>
     </row>
     <row r="120" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A120" s="10">
@@ -3012,7 +3012,7 @@
       <c r="D120" s="11">
         <v>495</v>
       </c>
-      <c r="E120" s="27"/>
+      <c r="E120" s="33"/>
     </row>
     <row r="121" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A121" s="10">
@@ -3027,7 +3027,7 @@
       <c r="D121" s="11">
         <v>495</v>
       </c>
-      <c r="E121" s="27"/>
+      <c r="E121" s="33"/>
     </row>
     <row r="122" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A122" s="10">
@@ -3042,7 +3042,7 @@
       <c r="D122" s="11">
         <v>495</v>
       </c>
-      <c r="E122" s="27"/>
+      <c r="E122" s="33"/>
     </row>
     <row r="123" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A123" s="10">
@@ -3057,7 +3057,7 @@
       <c r="D123" s="11">
         <v>495</v>
       </c>
-      <c r="E123" s="27"/>
+      <c r="E123" s="33"/>
     </row>
     <row r="124" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A124" s="10">
@@ -3072,7 +3072,7 @@
       <c r="D124" s="11">
         <v>495</v>
       </c>
-      <c r="E124" s="27"/>
+      <c r="E124" s="33"/>
     </row>
     <row r="125" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A125" s="10">
@@ -3087,7 +3087,7 @@
       <c r="D125" s="11">
         <v>495</v>
       </c>
-      <c r="E125" s="27"/>
+      <c r="E125" s="33"/>
     </row>
     <row r="126" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A126" s="10">
@@ -3102,7 +3102,7 @@
       <c r="D126" s="11">
         <v>495</v>
       </c>
-      <c r="E126" s="27"/>
+      <c r="E126" s="33"/>
     </row>
     <row r="127" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A127" s="10">
@@ -3117,7 +3117,7 @@
       <c r="D127" s="11">
         <v>495</v>
       </c>
-      <c r="E127" s="27"/>
+      <c r="E127" s="33"/>
     </row>
     <row r="128" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A128" s="10">
@@ -3132,7 +3132,7 @@
       <c r="D128" s="11">
         <v>495</v>
       </c>
-      <c r="E128" s="27"/>
+      <c r="E128" s="33"/>
     </row>
     <row r="129" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A129" s="10">
@@ -3147,7 +3147,7 @@
       <c r="D129" s="11">
         <v>1325</v>
       </c>
-      <c r="E129" s="27"/>
+      <c r="E129" s="33"/>
     </row>
     <row r="130" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A130" s="10">
@@ -3162,7 +3162,7 @@
       <c r="D130" s="11">
         <v>495</v>
       </c>
-      <c r="E130" s="27"/>
+      <c r="E130" s="33"/>
     </row>
     <row r="131" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A131" s="10">
@@ -3177,7 +3177,7 @@
       <c r="D131" s="11">
         <v>495</v>
       </c>
-      <c r="E131" s="27"/>
+      <c r="E131" s="33"/>
     </row>
     <row r="132" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A132" s="10">
@@ -3192,7 +3192,7 @@
       <c r="D132" s="11">
         <v>11380</v>
       </c>
-      <c r="E132" s="27"/>
+      <c r="E132" s="33"/>
     </row>
     <row r="133" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A133" s="10">
@@ -3207,7 +3207,7 @@
       <c r="D133" s="11">
         <v>495</v>
       </c>
-      <c r="E133" s="27"/>
+      <c r="E133" s="33"/>
     </row>
     <row r="134" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A134" s="10">
@@ -3222,7 +3222,7 @@
       <c r="D134" s="11">
         <v>495</v>
       </c>
-      <c r="E134" s="27"/>
+      <c r="E134" s="33"/>
     </row>
     <row r="135" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A135" s="10">
@@ -3237,7 +3237,7 @@
       <c r="D135" s="11">
         <v>1485</v>
       </c>
-      <c r="E135" s="27"/>
+      <c r="E135" s="33"/>
     </row>
     <row r="136" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A136" s="10">
@@ -3252,7 +3252,7 @@
       <c r="D136" s="11">
         <v>495</v>
       </c>
-      <c r="E136" s="27"/>
+      <c r="E136" s="33"/>
     </row>
     <row r="137" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A137" s="10">
@@ -3267,7 +3267,7 @@
       <c r="D137" s="11">
         <v>990</v>
       </c>
-      <c r="E137" s="27"/>
+      <c r="E137" s="33"/>
     </row>
     <row r="138" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A138" s="10">
@@ -3282,7 +3282,7 @@
       <c r="D138" s="11">
         <v>495</v>
       </c>
-      <c r="E138" s="27"/>
+      <c r="E138" s="33"/>
     </row>
     <row r="139" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A139" s="10">
@@ -3404,26 +3404,26 @@
       <c r="E146" s="17"/>
     </row>
     <row r="147" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="25" t="s">
+      <c r="A147" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="B147" s="25"/>
+      <c r="B147" s="31"/>
       <c r="C147" s="5"/>
-      <c r="D147" s="25" t="s">
+      <c r="D147" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="E147" s="25"/>
+      <c r="E147" s="31"/>
     </row>
     <row r="148" spans="1:5" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="26" t="s">
+      <c r="A148" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B148" s="26"/>
+      <c r="B148" s="32"/>
       <c r="C148" s="7"/>
-      <c r="D148" s="26" t="s">
+      <c r="D148" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="E148" s="26"/>
+      <c r="E148" s="32"/>
     </row>
     <row r="149" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A149" s="5"/>
@@ -3461,11 +3461,11 @@
       <c r="E153" s="5"/>
     </row>
     <row r="154" spans="1:5" s="2" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="25"/>
-      <c r="B154" s="25"/>
+      <c r="A154" s="31"/>
+      <c r="B154" s="31"/>
       <c r="C154" s="5"/>
-      <c r="D154" s="25"/>
-      <c r="E154" s="25"/>
+      <c r="D154" s="31"/>
+      <c r="E154" s="31"/>
     </row>
     <row r="155" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="156" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -3486,12 +3486,6 @@
   </sheetData>
   <autoFilter ref="A11:D145" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <mergeCells count="14">
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A1:B4"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="D147:E147"/>
     <mergeCell ref="A147:B147"/>
@@ -3500,6 +3494,12 @@
     <mergeCell ref="D148:E148"/>
     <mergeCell ref="D154:E154"/>
     <mergeCell ref="E12:E138"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A1:B4"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.25" top="1" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>